<commit_message>
Add a source-organism breakdown to the tracker's Summary tab
Bacteria, Archaea, Yeast/fungi, Plants, Viruses, Human, and the one
animal-derived outlier (a camelid nanobody), each with dataset/variant/paper
counts computed straight from every dataset's source_organism field. Datasets
and variants reconcile exactly against the Curated tab's totals.
</commit_message>
<xml_diff>
--- a/FitnessBench_2025_literature_search.xlsx
+++ b/FitnessBench_2025_literature_search.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +35,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -94,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -107,13 +111,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -485,12 +495,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -512,6 +524,8 @@
         </is>
       </c>
       <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -576,150 +590,381 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Sweep</t>
+          <t>Source-organism category</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>What it searched</t>
+          <t>Datasets</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Venue coverage</t>
+          <t>Variants</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Papers</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Example proteins</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>First sweep</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>"machine learning guided enzyme engineering" (+/- organism)</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>nature.com, 2025</t>
+          <t>Bacteria</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>93517</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>SpCas9 (PAMmla), RbcL, McbA, CjPglB, LbCas12a, creatinase</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Second sweep</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Same query, organism clause dropped</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Springer Nature via Europe PMC, 2025</t>
+          <t>Archaea</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>1753</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>ParLQ, PylRS (IFRS), pCNFRS, Tgo-D4K polymerase</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Third sweep</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>"deep mutational scanning" / "variant effect map" / "massively parallel mutagenesis" / "site-saturation mutagenesis"</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>All publishers via Europe PMC, 2025, open access</t>
+          <t>Yeast / fungi</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>118603</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>RNA Pol II Rpb1 (S. cerevisiae)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Fourth sweep (ACS)</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Title/abstract screen</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>ACS Catal, ACS Cent Sci, ACS Synth Biol, JACS, Biochemistry, 2025</t>
+          <t>Plants</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>419</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>AtHMT, CONSTANS (A. thaliana)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Fifth sweep (PNAS)</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Title-matched + abstract-matched protein/enzyme engineering terms</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>PNAS, 2025, open access</t>
+          <t>Viruses (incl. bacteriophage)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>270545</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>TEV protease, influenza NEP, T7 RNA polymerase, Con1 (designed potyviral consensus)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Sixth sweep (Cell Press)</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Title-matched</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Cell, Mol Cell, Cell Chem Biol, Cell Systems, Structure, Cell Host &amp; Microbe, Immunity, Curr Biol, Chem, iScience, Cell Rep Methods, Cell Rep Phys Sci</t>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>61070</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>MET kinase domain, SHP2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>Other (animal-derived)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>VHH nanobody, camelid-derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Subtotal: Prokaryotes (Bacteria + Archaea)</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>95270</v>
+      </c>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Subtotal: Eukaryotes, non-human (Yeast/fungi + Plants + Other)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>119080</v>
+      </c>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B21" s="7">
+        <f>SUM(B12:B18)</f>
+        <v/>
+      </c>
+      <c r="C21" s="7">
+        <f>SUM(C12:C18)</f>
+        <v/>
+      </c>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>'Papers' counts distinct DOIs within that category; a paper spanning several organisms (e.g. Jiang 2024/PRIME, which has datasets on a bacterium, an archaeon, a bacteriophage and a camelid nanobody) is counted once per category it touches, so the Papers column does not sum to 16. Datasets and Variants do sum exactly to the Curated tab's totals -- every dataset has exactly one source_organism. 'Other (animal-derived)' is the VHH nanobody dataset, filed under datasets/ even though a camelid is not a bacterium, archaeon, yeast or plant -- the branch has no separate tree for it yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Sweep</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>What it searched</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Venue coverage</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>First sweep</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>"machine learning guided enzyme engineering" (+/- organism)</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>nature.com, 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Second sweep</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Same query, organism clause dropped</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Springer Nature via Europe PMC, 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Third sweep</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>"deep mutational scanning" / "variant effect map" / "massively parallel mutagenesis" / "site-saturation mutagenesis"</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>All publishers via Europe PMC, 2025, open access</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Fourth sweep (ACS)</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Title/abstract screen</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>ACS Catal, ACS Cent Sci, ACS Synth Biol, JACS, Biochemistry, 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Fifth sweep (PNAS)</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Title-matched + abstract-matched protein/enzyme engineering terms</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>PNAS, 2025, open access</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Sixth sweep (Cell Press)</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Title-matched</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Cell, Mol Cell, Cell Chem Biol, Cell Systems, Structure, Cell Host &amp; Microbe, Immunity, Curr Biol, Chem, iScience, Cell Rep Methods, Cell Rep Phys Sci</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>"directed evolution" / "site-saturation mutagenesis" / "laboratory evolution" / "yeast surface display"+"deep sequencing", explicitly excluding "deep mutational scanning" and "enzyme engineering" phrasing</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>All publishers via Europe PMC, 2025, journals only (no bioRxiv)</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="33" ht="45" customHeight="1">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>See the 'Curated' tab for shipped datasets with variant counts, 'Rejected' for every paper chased to a documented reason, and 'Open (maybes)' for leads left for a future session. Full narrative detail, including access routes and per-sweep notes, is in candidates_2025.md on the 2025 branch.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A20:C20"/>
+  <mergeCells count="3">
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A33:E33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -799,711 +1044,711 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="n">
+      <c r="A2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Zhang</t>
         </is>
       </c>
-      <c r="C2" s="7" t="n">
+      <c r="C2" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>Nat Commun</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>Machine learning-guided evolution of pyrrolysyl-tRNA synthetase for improved incorporation efficiency of diverse noncanonical amino acids</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-61952-2</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
         <is>
           <t>datasets</t>
         </is>
       </c>
-      <c r="H2" s="7" t="n">
+      <c r="H2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="7" t="n">
+      <c r="I2" s="9" t="n">
         <v>508</v>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="9" t="inlineStr">
         <is>
           <t>IFRS (PylRS variant); FFT-PLSR-guided rounds rebased onto one scale</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="n">
+      <c r="A3" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Huber</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n">
+      <c r="C3" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Nat Commun</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Data-driven protease engineering by DNA-recording and epistasis-aware machine learning</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-60622-7</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>datasets_virus</t>
         </is>
       </c>
-      <c r="H3" s="7" t="n">
+      <c r="H3" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="I3" s="7" t="n">
+      <c r="I3" s="9" t="n">
         <v>268446</v>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="J3" s="9" t="inlineStr">
         <is>
           <t>TEV protease (MLDEEP); one dataset per P1' substrate residue plus a full saturation scan</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="n">
+      <c r="A4" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Duan</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Nat Commun</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Widespread epistasis shapes RNA polymerase II active site function and evolution</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-63304-6</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>datasets</t>
         </is>
       </c>
-      <c r="H4" s="7" t="n">
+      <c r="H4" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="I4" s="7" t="n">
+      <c r="I4" s="9" t="n">
         <v>118603</v>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>RNA Pol II Rpb1 trigger loop, S. cerevisiae; growth fitness across selective conditions</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Landwehr</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Nat Commun</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Accelerated enzyme engineering by machine-learning guided cell-free expression</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>10.1038/s41467-024-55399-0</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>datasets</t>
         </is>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="H5" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="I5" s="7" t="n">
+      <c r="I5" s="9" t="n">
         <v>10909</v>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="J5" s="9" t="inlineStr">
         <is>
           <t>McbA amide synthetase; conversion of 9 pharmaceuticals</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Yang</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Nat Commun</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Active learning-assisted directed evolution</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-55987-8</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>datasets</t>
         </is>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="I6" s="9" t="n">
         <v>790</v>
       </c>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>ParLQ; diastereoselectivity and yield on a non-native cyclopropanation (ALDE)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Singh</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Nat Commun</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>A generalized platform for artificial intelligence-powered autonomous enzyme engineering</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-61209-y</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>datasets</t>
         </is>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="7" t="n">
+      <c r="I7" s="9" t="n">
         <v>176</v>
       </c>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="J7" s="9" t="inlineStr">
         <is>
           <t>AtHMT methyltransferase, substrate preference</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Zhang</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Nat Commun</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>Integrating protein language models and automatic biofoundry for enhanced protein evolution</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-56751-8</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>datasets</t>
         </is>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="7" t="n">
+      <c r="I8" s="9" t="n">
         <v>384</v>
       </c>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="J8" s="9" t="inlineStr">
         <is>
           <t>pCNFRS tRNA synthetase; 4 rounds of ESM-2-nominated variants</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Silverstein</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Nature</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>Custom CRISPR-Cas9 PAM variants via scalable engineering and machine learning</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>10.1038/s41586-025-09021-y</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>datasets</t>
         </is>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="H9" s="9" t="n">
         <v>64</v>
       </c>
-      <c r="I9" s="7" t="n">
+      <c r="I9" s="9" t="n">
         <v>68992</v>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J9" s="9" t="inlineStr">
         <is>
           <t>PAMmla; ~1,078 SpCas9 variants per dataset, PAM specificity</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Alamos</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Nat Biotechnol</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Multiplexed profiling of transcriptional regulators in plant cells</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>10.1038/s41587-025-02880-w</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>datasets</t>
         </is>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="7" t="n">
+      <c r="I10" s="9" t="n">
         <v>243</v>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="J10" s="9" t="inlineStr">
         <is>
           <t>CONSTANS activation domain (ENTRAP-seq); tile libraries out of scope, single-substitution table only</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Jiang</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="9" t="n">
         <v>2024</v>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Sci Adv</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>A general temperature-guided language model to design proteins of enhanced stability and activity</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>10.1126/sciadv.adr2641</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>datasets + datasets_virus</t>
         </is>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="H11" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="I11" s="7" t="n">
+      <c r="I11" s="9" t="n">
         <v>353</v>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="J11" s="9" t="inlineStr">
         <is>
           <t>PRIME platform; Tgo-D4K polymerase, VHH nanobody, LbCas12a, creatinase, T7 RNA polymerase</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Estevam</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>eLife</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>Mapping kinase domain resistance mechanisms for the MET receptor tyrosine kinase via deep mutational scanning</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>10.7554/eLife.101882</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>datasets_human</t>
         </is>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="H12" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="I12" s="7" t="n">
+      <c r="I12" s="9" t="n">
         <v>44889</v>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="J12" s="9" t="inlineStr">
         <is>
           <t>MET kinase domain; one dataset per inhibitor plus DMSO control</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Jiang</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Nat Commun</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Deep mutational scanning of the multi-domain phosphatase SHP2 reveals mechanisms of regulation and pathogenicity</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-60641-4</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>datasets_human</t>
         </is>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="H13" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="I13" s="7" t="n">
+      <c r="I13" s="9" t="n">
         <v>16181</v>
       </c>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="J13" s="9" t="inlineStr">
         <is>
           <t>SHP2 full-length and isolated PTP domain; yeast growth-rescue enrichment</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Wysocki</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="9" t="n">
         <v>2026</v>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>ACS Synth Biol</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>High-Throughput Detection of Cyanobacterial Form I Rubisco Assembly</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>10.1021/acssynbio.5c00591</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
         <is>
           <t>datasets</t>
         </is>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="H14" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="I14" s="7" t="n">
+      <c r="I14" s="9" t="n">
         <v>13216</v>
       </c>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="J14" s="9" t="inlineStr">
         <is>
           <t>RbcL (H. neapolitanus); phage-selection site-saturation, with/without GroELS</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Thornton</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>ACS Synth Biol</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>Cell-Free Protein Synthesis as a Method to Rapidly Screen Machine Learning-Generated Protease Variants</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>10.1021/acssynbio.5c00062</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>datasets_virus</t>
         </is>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="I15" s="7" t="n">
+      <c r="I15" s="9" t="n">
         <v>96</v>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J15" s="9" t="inlineStr">
         <is>
           <t>Con1, a designed consensus potyviral protease; region A and B site-saturation</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Teo</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Cell Rep</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>Probing the functional constraints of influenza A virus NEP by deep mutational scanning</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>10.1016/j.celrep.2024.115196</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>datasets_virus</t>
         </is>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="H16" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="I16" s="7" t="n">
+      <c r="I16" s="9" t="n">
         <v>1894</v>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="J16" s="9" t="inlineStr">
         <is>
           <t>Influenza A NEP, A/WSN/1933 strain; found via title sweep, data was on Zenodo not in the article supplement</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Wong</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Nat Commun</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>Characterizing and engineering post-translational modifications with high-throughput cell-free expression</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-60526-6</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>datasets</t>
         </is>
       </c>
-      <c r="H17" s="7" t="n">
+      <c r="H17" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="7" t="n">
+      <c r="I17" s="9" t="n">
         <v>285</v>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J17" s="9" t="inlineStr">
         <is>
           <t>CjPglB oligosaccharyltransferase; 15-position site-saturation, AlphaLISA glycosylation signal</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -1514,11 +1759,11 @@
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
-      <c r="H18" s="8">
+      <c r="H18" s="10">
         <f>SUM(H2:H17)</f>
         <v/>
       </c>
-      <c r="I18" s="8">
+      <c r="I18" s="10">
         <f>SUM(I2:I17)</f>
         <v/>
       </c>
@@ -1573,1350 +1818,1350 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="n">
+      <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>iCASE 2025, thermostability/activity tailoring</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-55944-5</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Second sweep</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>No work item reaches the 20-variant floor. 63-sheet Source Data workbook; every sheet with mutant labels holds at most 16 rows; the large sheets are simulation output (DSI, compressibility, binding free energy), not experimental measurement.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="n">
+      <c r="A3" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Artificial metathase (de novo + directed evolution)</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41929-025-01436-0</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>Second sweep</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>No variant table. One spreadsheet per figure, 4-38 rows each of kinetics/titration data, none a per-variant list.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n">
+      <c r="A4" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Kemp eliminase distal mutations (3 de novo enzymes)</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-63802-7</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>Second sweep</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>No variant table. Four sheets of kinetic traces / stopped-flow raw data, no mutant-labelled block.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>ML prediction-tool papers evaluated on others' data (CatPred, CataPro, TopEC, PreMode, DeepMVP, ABACUS-T, LassoESM, cross-attention specificity GNN, biophysics-based PLMs)</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>(various, not individually recorded)</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>Second sweep</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>Phase 1 exclusion: a dataset a paper merely evaluates on belongs to whoever measured it, not to the modeling paper.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>AI-designed base/prime editors</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41586-025-09298-z</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>Second sweep</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>AI-designed editors are not variants of one wild type.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Reviews/perspectives bundle (ML applied to biocatalysis, PET hydrolase standardisation guidelines, C1 utilisation)</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>(not recorded)</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>Second sweep</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>Reviews, not primary measurement papers.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="n">
+      <c r="A8" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>DMS in E. coli periplasm (human A-beta-42 amyloid propensity)</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>10.1073/pnas.2516165122</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>Third sweep</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Assay host is bacterial but the protein is human (A-beta-42); readout is aggregation propensity via a bacterial reporter, not enzyme fitness. Deprioritized to datasets_human/ scope, not chased further.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n">
+      <c r="A9" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Reshaping a glycoside hydrolase active site (330,000-clone droplet sort)</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>10.1021/acscentsci.5c01227</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>Third sweep</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>Only a handful of named winners (M1, M2, ...) individually characterised; no systematic per-variant table in the paper or its PDF-only supplement.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="n">
+      <c r="A10" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Deep Mutational Scanning of FDX1</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-67869-0</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>Third sweep</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>FigShare deposit holds only raw Enrich2-style per-sample counts (2.1 GB), not scores. Source Data has only anonymized score distributions and position-averaged values, no per-variant readout.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n">
+      <c r="A11" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>EGFR resistance to 4th-generation TKIs</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41698-025-01086-2</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>Third sweep</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>Same experimental shape as the curated MET paper, but no GitHub deposit. Data availability names only raw GEO reads; the PDF-only supplement holds FEP calculations for a handful of representative isoforms, not a per-variant table.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="n">
+      <c r="A12" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Glucokinase variant characterization</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>10.3390/ijms27010156</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>Third sweep</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>25 individually chosen clinical variants, well under the floor; not a saturation library.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="n">
+      <c r="A13" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Directed evolution of a beta-lactamase (conformational states)</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>10.1002/pro.70322</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>Third sweep</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>3 successive mutants + WT, well under the floor.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="n">
+      <c r="A14" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Deep structure-function analysis of Mus81 (dominant mutational scanning)</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>10.1073/pnas.2506043122</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>Third sweep</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Deposited data is a binary Y/N hit classification (dominant / fails-to-complement), not a quantitative per-variant score; graded growth-sensitivity data not deposited.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="n">
+      <c r="A15" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Pyranose oxidase oligomerization engineering</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>10.1111/febs.70004</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>Third sweep</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>Zenodo deposit is models/docking scores only; experimental data available upon request.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="n">
+      <c r="A16" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Isophthalate dioxygenase engineering</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>10.1128/jb.00221-25</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Third sweep</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>No data-availability statement found.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="n">
+      <c r="A17" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Confocal absorbance-activated droplet sorting (cAADS)</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>10.1002/advs.202505324</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Third sweep</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>Data available from the corresponding author upon reasonable request.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="n">
+      <c r="A18" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Directed evolution of a plant Rubisco chaperone</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>10.1073/pnas.2510701122</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>Third + fifth sweep</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>PDF-only SI; text says 'selected' variants, not a full library table.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="n">
+      <c r="A19" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>In vivo directed evolution of an ultrafast Rubisco</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>10.1073/pnas.2505083122</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Third + fifth sweep</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>Kinetic characterisation covers only ~7 named substitutions; the 292-row dataset is population allele-frequency trajectories per locus across evolution rounds, not per-clone genotype-fitness pairs.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="n">
+      <c r="A20" s="11" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Directed evolution of a covalent RNA-labeling tag</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>10.1073/pnas.2422085122</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>Third + fifth sweep</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>PDF-only SI.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="n">
+      <c r="A21" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Nanobody-antigen interface optimisation</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>10.1073/pnas.2426438122</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>Third + fifth sweep</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>PDF-only SI; phage display down to a small validated set.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="n">
+      <c r="A22" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>PET hydrolases from natural diversity</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>(not recorded)</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>Fourth sweep (ACS)</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Homolog panel of ~400 distinct natural sequences, no shared wild type.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="n">
+      <c r="A23" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>KdcA directed evolution</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>(not recorded)</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>Fourth sweep (ACS)</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>PDF-only supplement; text names one 8-substitution final variant, not a library table.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="n">
+      <c r="A24" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>DyP peroxidase thermostability</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>(not recorded)</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>Fourth sweep (ACS)</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>PDF-only supplement, a handful of designed variants.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="n">
+      <c r="A25" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>SPOT metallopeptide library</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>(not recorded)</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Fourth sweep (ACS)</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>PDF-only supplement, small named set.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="n">
+      <c r="A26" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>F. rodentium Cas9 (structural/cryo-EM)</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>(not recorded)</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>Sixth sweep (Cell Press)</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Not chased further -- likely a handful of validated point mutants, no data-availability statement found.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="n">
+      <c r="A27" s="11" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>ODM protein-design pipeline</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>(not recorded)</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>Sixth sweep (Cell Press)</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>Not chased further -- generative-model paper, likely benchmarks on public data (Phase 1 evaluated-on exclusion).</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="n">
+      <c r="A28" s="11" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>Chen 2025, Cas12a variant profiling</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-57150-9</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>'Variants' are 24 orthologs, and activity varies per target sequence, not per protein substitution -- no single wild-type to normalise against.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="n">
+      <c r="A29" s="11" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Zhu 2025, DropAI droplet screening</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-58139-0</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>ML optimises the cell-free reaction composition, not protein sequence.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="n">
+      <c r="A30" s="11" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>m6A-IIN modification-site prediction</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>10.1038/s42003-025-08265-8</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>RNA modification sites, no protein variants.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="n">
+      <c r="A31" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Nanozymes review</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-62063-8</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>Review.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="n">
+      <c r="A32" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>CRISPR-Cas in agriculture</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41580-025-00834-3</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E32" s="9" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Review.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="n">
+      <c r="A33" s="11" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>CRISPR single-nucleotide diagnostics</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>10.1038/s43856-025-00933-4</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E33" s="11" t="inlineStr">
         <is>
           <t>Review.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="n">
+      <c r="A34" s="11" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>One-carbon biochemicals</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>10.1038/s44160-025-00835-2</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Review.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="n">
+      <c r="A35" s="11" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>Antimicrobial peptides</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41579-025-01200-y</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D35" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E35" s="11" t="inlineStr">
         <is>
           <t>Review.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="n">
+      <c r="A36" s="11" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>Protein folding and proteostasis</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41392-025-02439-w</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Review.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="n">
+      <c r="A37" s="11" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>Non-CG DNA methylation</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41588-025-02303-1</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="D37" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E37" s="11" t="inlineStr">
         <is>
           <t>Review.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="n">
+      <c r="A38" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Antibacterial preclinical pipeline</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41579-025-01167-w</t>
         </is>
       </c>
-      <c r="D38" s="9" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E38" s="9" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Review.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="9" t="n">
+      <c r="A39" s="11" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>African bioeconomy genomics</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>10.1038/s44185-025-00102-9</t>
         </is>
       </c>
-      <c r="D39" s="9" t="inlineStr">
+      <c r="D39" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="E39" s="11" t="inlineStr">
         <is>
           <t>Perspective.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="9" t="n">
+      <c r="A40" s="11" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="9" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>Seven technologies to watch in 2025</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>10.1038/d41586-025-00075-6</t>
         </is>
       </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="D40" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E40" s="9" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>News feature.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="9" t="n">
+      <c r="A41" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>ESHG 2025 ePoster abstracts</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41431-025-01934-6</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D41" s="11" t="inlineStr">
         <is>
           <t>Rejected list (early sweeps)</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E41" s="11" t="inlineStr">
         <is>
           <t>Conference abstracts.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="n">
+      <c r="A42" s="11" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="9" t="inlineStr">
+      <c r="B42" s="11" t="inlineStr">
         <is>
           <t>Wong (chitosanase, signal peptide optimization)</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr">
+      <c r="C42" s="11" t="inlineStr">
         <is>
           <t>10.1021/acs.jafc.5c13730</t>
         </is>
       </c>
-      <c r="D42" s="9" t="inlineStr">
+      <c r="D42" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E42" s="9" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Iterative rounds to one named winner (M8); paywalled, not opened past the abstract.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="9" t="n">
+      <c r="A43" s="11" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>PROTEUS mammalian directed-evolution platform</t>
         </is>
       </c>
-      <c r="C43" s="9" t="inlineStr">
+      <c r="C43" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41467-025-59438-2</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D43" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E43" s="9" t="inlineStr">
+      <c r="E43" s="11" t="inlineStr">
         <is>
           <t>Methods/tool paper; the 'N variants' figures are allele-frequency spectra from continuous passaging, not an isolated-clone table; the two characterized Nb139 mutations are far under floor.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="9" t="n">
+      <c r="A44" s="11" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="9" t="inlineStr">
+      <c r="B44" s="11" t="inlineStr">
         <is>
           <t>Golden Gate continuous-evolution toolkit</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
+      <c r="C44" s="11" t="inlineStr">
         <is>
           <t>10.1093/synbio/ysaf014</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr">
+      <c r="D44" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E44" s="9" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Pure toolkit demonstration; no target-protein dataset, just proof the mutator works.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="9" t="n">
+      <c r="A45" s="11" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="9" t="inlineStr">
+      <c r="B45" s="11" t="inlineStr">
         <is>
           <t>Maize HPPD via TADR</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
+      <c r="C45" s="11" t="inlineStr">
         <is>
           <t>10.1111/pbi.70160</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr">
+      <c r="D45" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E45" s="9" t="inlineStr">
+      <c r="E45" s="11" t="inlineStr">
         <is>
           <t>3-page technical advance; 9 point mutants individually tested, qualitative colony-color readout for most.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="9" t="n">
+      <c r="A46" s="11" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="9" t="inlineStr">
+      <c r="B46" s="11" t="inlineStr">
         <is>
           <t>MerR Hg2+ biosensor</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
+      <c r="C46" s="11" t="inlineStr">
         <is>
           <t>10.1016/j.bios.2025.117687</t>
         </is>
       </c>
-      <c r="D46" s="9" t="inlineStr">
+      <c r="D46" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E46" s="9" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Selection funnel (98% eliminated, then top 0.2%) ending in one named variant (V124E); not open access.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="9" t="n">
+      <c r="A47" s="11" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="9" t="inlineStr">
+      <c r="B47" s="11" t="inlineStr">
         <is>
           <t>Oncolytic Sindbis virus (osteosarcoma)</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
+      <c r="C47" s="11" t="inlineStr">
         <is>
           <t>10.1016/j.omton.2025.201096</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="D47" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E47" s="11" t="inlineStr">
         <is>
           <t>Adaptive passaging to a consensus lineage, not a mapped substitution landscape; 'variant' appears 6 times in the whole paper.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="9" t="n">
+      <c r="A48" s="11" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="9" t="inlineStr">
+      <c r="B48" s="11" t="inlineStr">
         <is>
           <t>Rubisco laboratory-evolution screen (Nat Plants)</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
+      <c r="C48" s="11" t="inlineStr">
         <is>
           <t>10.1038/s41477-025-02093-8</t>
         </is>
       </c>
-      <c r="D48" s="9" t="inlineStr">
+      <c r="D48" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E48" s="9" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Screen narrows to exactly two named point mutations (M116L, A242V), deeply characterized but not a library table.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="9" t="n">
+      <c r="A49" s="11" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="9" t="inlineStr">
+      <c r="B49" s="11" t="inlineStr">
         <is>
           <t>Nonheme iron BsQueD (alkene amination)</t>
         </is>
       </c>
-      <c r="C49" s="9" t="inlineStr">
+      <c r="C49" s="11" t="inlineStr">
         <is>
           <t>10.1021/jacsau.5c00817</t>
         </is>
       </c>
-      <c r="D49" s="9" t="inlineStr">
+      <c r="D49" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E49" s="9" t="inlineStr">
+      <c r="E49" s="11" t="inlineStr">
         <is>
           <t>'An optimized variant' -- lineage evolution to one champion.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="9" t="n">
+      <c r="A50" s="11" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="9" t="inlineStr">
+      <c r="B50" s="11" t="inlineStr">
         <is>
           <t>PchB to chorismate mutase (reverse evolution)</t>
         </is>
       </c>
-      <c r="C50" s="9" t="inlineStr">
+      <c r="C50" s="11" t="inlineStr">
         <is>
           <t>10.1021/acs.biochem.5c00157</t>
         </is>
       </c>
-      <c r="D50" s="9" t="inlineStr">
+      <c r="D50" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E50" s="9" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Functional-complementation selection from a 7-position, 38,000-variant library down to a handful of named sequenced clones; no per-variant table, just individually characterized survivors.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="n">
+      <c r="A51" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="9" t="inlineStr">
+      <c r="B51" s="11" t="inlineStr">
         <is>
           <t>PHL7 PET hydrolase (4 rounds)</t>
         </is>
       </c>
-      <c r="C51" s="9" t="inlineStr">
+      <c r="C51" s="11" t="inlineStr">
         <is>
           <t>10.1016/j.checat.2025.101399</t>
         </is>
       </c>
-      <c r="D51" s="9" t="inlineStr">
+      <c r="D51" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E51" s="9" t="inlineStr">
+      <c r="E51" s="11" t="inlineStr">
         <is>
           <t>Four named final variants (Jemez, Santa Fe, Taos, Tusas); no deposited dataset, 'available upon reasonable request'.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="9" t="n">
+      <c r="A52" s="11" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="9" t="inlineStr">
+      <c r="B52" s="11" t="inlineStr">
         <is>
           <t>Q-body immunosensor quenching prediction</t>
         </is>
       </c>
-      <c r="C52" s="9" t="inlineStr">
+      <c r="C52" s="11" t="inlineStr">
         <is>
           <t>10.1021/jacsau.4c01189</t>
         </is>
       </c>
-      <c r="D52" s="9" t="inlineStr">
+      <c r="D52" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E52" s="9" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>The large NGS-scored library is a synthetic nanobody repertoire, not point mutants of one wild type; validated point-mutant sets (Trp scans) are single digits per antibody.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="n">
+      <c r="A53" s="11" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="9" t="inlineStr">
+      <c r="B53" s="11" t="inlineStr">
         <is>
           <t>Curr Protoc SELIS walkthrough</t>
         </is>
       </c>
-      <c r="C53" s="9" t="inlineStr">
+      <c r="C53" s="11" t="inlineStr">
         <is>
           <t>10.1002/cpz1.70218</t>
         </is>
       </c>
-      <c r="D53" s="9" t="inlineStr">
+      <c r="D53" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E53" s="9" t="inlineStr">
+      <c r="E53" s="11" t="inlineStr">
         <is>
           <t>Protocol demonstration, not a dataset paper.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="9" t="n">
+      <c r="A54" s="11" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="9" t="inlineStr">
+      <c r="B54" s="11" t="inlineStr">
         <is>
           <t>Ebola VP40 patient mutations</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
+      <c r="C54" s="11" t="inlineStr">
         <is>
           <t>10.1016/j.jbc.2025.110489</t>
         </is>
       </c>
-      <c r="D54" s="9" t="inlineStr">
+      <c r="D54" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E54" s="9" t="inlineStr">
+      <c r="E54" s="11" t="inlineStr">
         <is>
           <t>'40 mutations' is epidemiological surveillance across outbreak lineages, not an experimental library; only 2 mutations (R204H, H269R) are lab-characterized.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="9" t="n">
+      <c r="A55" s="11" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="9" t="inlineStr">
+      <c r="B55" s="11" t="inlineStr">
         <is>
           <t>Affibody stability (DR5 / TNFR1)</t>
         </is>
       </c>
-      <c r="C55" s="9" t="inlineStr">
+      <c r="C55" s="11" t="inlineStr">
         <is>
           <t>10.1002/bit.28954</t>
         </is>
       </c>
-      <c r="D55" s="9" t="inlineStr">
+      <c r="D55" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E55" s="9" t="inlineStr">
+      <c r="E55" s="11" t="inlineStr">
         <is>
           <t>Deep sequencing used only to triage candidates for individual validation; reported data is a handful of purified variants, not library-wide.</t>
         </is>
@@ -2977,90 +3222,90 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="n">
+      <c r="A2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Class A beta-lactamase gatekeeper-residue screen (5 enzymes)</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>10.1016/j.jbc.2025.110347</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>Genuine deep-sequencing fitness data in a legacy .xls (needs xlrd): site saturation of Ambler position 105 in BlaC, CTX-M-14, KPC-2, NmcA, TEM-1, each vs. 7 substrates/inhibitors, 3 replicates, raw counts and per-replicate fitness values -- not just a figure.</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>Single saturated position per enzyme: 19 substitutions + WT, one row under this branch's usual floor. Worth a second look if the bar is 'genuine deep-sequencing data' rather than 'library-scale'.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="n">
+      <c r="A3" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Tryptophan decarboxylase (TDC) active-site recombination (SUMS)</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>10.1002/pro.70356</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>Substrate-multiplexed screening across 5 active-site positions; a clean prior single-site-saturation sub-library (96 unique single mutants) plus iterative combinatorial recombination libraries (~250 variants total, up to triple mutants, LC-MS-quantified). Multi-site labels are within format scope.</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>Data availability is 'upon reasonable request' -- nothing machine-readable found in the supplement. Needs an email to the authors.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="n">
+      <c r="A4" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Yeast-display A-beta-fibril conformational antibody campaign</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>10.3389/fimmu.2025.1655893</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>Real NGS sort-round data deposited on GitHub (Tessier-Lab-UMich/druglike-abeta-antibodies): CDR-sequence frequency tables for a defined 10-site NNK library (5 in HCDR1, 5 in LCDR2) built off a named parent antibody ('clone 97').</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>Needs clone 97's parent CDR sequence from a different, earlier paper, and working out which numbered file per replicate is 'before' vs. 'after' selection -- not safe to guess at.</t>
         </is>

</xml_diff>

<commit_message>
Make the sweep table in the Summary tab specific, especially sweep four
Sweep four (ACS) never had a recorded boolean query in candidates_2025.md,
unlike the others -- it was a direct browse-and-read pass, not a single
search string, and that's now stated plainly instead of glossed over as
"title/abstract screen". Also added the hit counts for sweeps five and six
that were already on record but not carried into the spreadsheet.
</commit_message>
<xml_diff>
--- a/FitnessBench_2025_literature_search.xlsx
+++ b/FitnessBench_2025_literature_search.xlsx
@@ -893,12 +893,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Title/abstract screen</t>
+          <t>No single boolean query recorded (unlike the other sweeps) -- browsed each journal's 2025 issue listings directly, then read title and abstract of anything protein/enzyme-shaped. Direct ACS access returns a 403 on articles and supplements, so retrieval for anything that looked promising went through Europe PMC instead.</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>ACS Catal, ACS Cent Sci, ACS Synth Biol, JACS, Biochemistry, 2025</t>
+          <t>ACS Catal, ACS Cent Sci, ACS Synth Biol, JACS, Biochemistry, 2025, open access</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Title-matched + abstract-matched protein/enzyme engineering terms</t>
+          <t>Two separate matches, then deduped: title-matched on protein/enzyme-engineering terms (30 hits) and abstract-matched on landscape/library terms ("fitness landscape", "combinatorial library", etc., 11 hits) -- 41 unique papers total.</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Title-matched</t>
+          <t>Title-matched across the full journal family (43 hits) -- almost entirely clinical-ML iScience papers with no connection to protein engineering, so no separate abstract pass was run.</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Update the tracker for the redone ACS sweep
Adds Somvilla 2025 (8 datasets, 160 variants), the four new rejections, and
the seventh sweep's row. Marks the fourth sweep SUPERSEDED rather than
deleting it -- it is the reason the seventh exists, and the contrast between
a manual browse and a real query is the useful part of the record.
</commit_message>
<xml_diff>
--- a/FitnessBench_2025_literature_search.xlsx
+++ b/FitnessBench_2025_literature_search.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>135</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6">
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>545965</v>
+        <v>546125</v>
       </c>
     </row>
     <row r="7">
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
@@ -621,17 +621,17 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>93517</v>
+        <v>93677</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>SpCas9 (PAMmla), RbcL, McbA, CjPglB, LbCas12a, creatinase</t>
+          <t>SpCas9 (PAMmla), RbcL, McbA, CjPglB, SaAmd, LbCas12a, creatinase</t>
         </is>
       </c>
     </row>
@@ -768,10 +768,10 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>95270</v>
+        <v>95430</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
@@ -811,7 +811,7 @@
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>'Papers' counts distinct DOIs within that category; a paper spanning several organisms (e.g. Jiang 2024/PRIME, which has datasets on a bacterium, an archaeon, a bacteriophage and a camelid nanobody) is counted once per category it touches, so the Papers column does not sum to 16. Datasets and Variants do sum exactly to the Curated tab's totals -- every dataset has exactly one source_organism. 'Other (animal-derived)' is the VHH nanobody dataset, filed under datasets/ even though a camelid is not a bacterium, archaeon, yeast or plant -- the branch has no separate tree for it yet.</t>
+          <t>'Papers' counts distinct DOIs within that category; a paper spanning several organisms (e.g. Jiang 2024/PRIME, which has datasets on a bacterium, an archaeon, a bacteriophage and a camelid nanobody) is counted once per category it touches, so the Papers column does not sum to the 17-paper total. Datasets and Variants do sum exactly to the Curated tab's totals -- every dataset has exactly one source_organism. 'Other (animal-derived)' is the VHH nanobody dataset, filed under datasets/ even though a camelid is not a bacterium, archaeon, yeast or plant -- the branch has no separate tree for it yet.</t>
         </is>
       </c>
     </row>
@@ -888,12 +888,12 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Fourth sweep (ACS)</t>
+          <t>Fourth sweep (ACS) -- SUPERSEDED</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>No single boolean query recorded (unlike the other sweeps) -- browsed each journal's 2025 issue listings directly, then read title and abstract of anything protein/enzyme-shaped. Direct ACS access returns a 403 on articles and supplements, so retrieval for anything that looked promising went through Europe PMC instead.</t>
+          <t>No single boolean query recorded (unlike the other sweeps) -- browsed each journal's 2025 issue listings directly, then read title and abstract of anything protein/enzyme-shaped. Direct ACS access returns a 403 on articles and supplements, so retrieval went through Europe PMC. Redone systematically as the seventh sweep below, which found a paper this pass missed.</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -939,22 +939,39 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
+          <t>Seventh sweep (ACS, redone)</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>The fourth sweep redone as a real query for parity with the others: JOURNAL:(5 ACS titles) AND PUB_YEAR:2025 AND SRC:MED AND (deep mutational scanning OR site-saturation mutagenesis OR directed evolution OR variant effect map OR massively parallel mutagenesis OR enzyme engineering OR protein engineering, as quoted phrases) -- 237 hits, 234 unseen; all 234 abstracts pulled and keyword-scored for per-variant-table signals. Found Somvilla 2025, which the manual pass had missed.</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>ACS Catal, ACS Cent Sci, ACS Synth Biol, JACS, Biochemistry, 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>"directed evolution" / "site-saturation mutagenesis" / "laboratory evolution" / "yeast surface display"+"deep sequencing", explicitly excluding "deep mutational scanning" and "enzyme engineering" phrasing</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>All publishers via Europe PMC, 2025, journals only (no bioRxiv)</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="45" customHeight="1">
-      <c r="A33" s="8" t="inlineStr">
+    <row r="34" ht="45" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>See the 'Curated' tab for shipped datasets with variant counts, 'Rejected' for every paper chased to a documented reason, and 'Open (maybes)' for leads left for a future session. Full narrative detail, including access routes and per-sweep notes, is in candidates_2025.md on the 2025 branch.</t>
         </is>
@@ -964,7 +981,7 @@
   <mergeCells count="3">
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A34:E34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -976,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1748,26 +1765,70 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Somvilla</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>ACS Catalysis</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Ultrahigh-Throughput Activity Engineering of Promiscuous Amidases through a Fluorescence-Activated Cell Sorting Assay</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.5c01903</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>datasets</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>160</v>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>SaAmd amidase (Sphingomonas alpina); one dataset per substrate across 8 amide/ester/carbamate substrates</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
-      <c r="H18" s="10">
-        <f>SUM(H2:H17)</f>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="10">
+        <f>SUM(H2:H18)</f>
         <v/>
       </c>
-      <c r="I18" s="10">
-        <f>SUM(I2:I17)</f>
+      <c r="I19" s="10">
+        <f>SUM(I2:I18)</f>
         <v/>
       </c>
-      <c r="J18" s="4" t="n"/>
+      <c r="J19" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1780,7 +1841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3148,20 +3209,120 @@
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
+          <t>Cyanobacterial screening platform for Rubisco mutant variants</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="inlineStr">
+        <is>
+          <t>10.1021/acssynbio.5c00065</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>Seventh sweep (ACS, redone)</t>
+        </is>
+      </c>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>16 variants, under the floor -- the authors' own GitHub repository is named CbbM_16variants. Deep-sequenced competitive growth, so the shape is right and only the size is wrong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>Ultrahigh-throughput multiplexed screening from cell-free expression</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>10.1021/jacs.5c04962</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Seventh sweep (ACS, redone)</t>
+        </is>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>Not open access, no PMC record; a droplet-microfluidics methods paper rather than a variant dataset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>Directed evolution of a genetically encoded chloride indicator</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="inlineStr">
+        <is>
+          <t>10.1021/acssynbio.4c00818</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>Seventh sweep (ACS, redone)</t>
+        </is>
+      </c>
+      <c r="E57" s="11" t="inlineStr">
+        <is>
+          <t>fullTextXML empty; abstract describes a lineage to a named improved indicator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>Stereoselective photoenzymatic hydroarylation</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>10.1021/jacs.5c12440</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Seventh sweep (ACS, redone)</t>
+        </is>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>fullTextXML empty; biocatalysis paper evolving to a named champion variant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
           <t>Affibody stability (DR5 / TNFR1)</t>
         </is>
       </c>
-      <c r="C55" s="11" t="inlineStr">
+      <c r="C59" s="11" t="inlineStr">
         <is>
           <t>10.1002/bit.28954</t>
         </is>
       </c>
-      <c r="D55" s="11" t="inlineStr">
+      <c r="D59" s="11" t="inlineStr">
         <is>
           <t>Directed-evolution sweep</t>
         </is>
       </c>
-      <c r="E55" s="11" t="inlineStr">
+      <c r="E59" s="11" t="inlineStr">
         <is>
           <t>Deep sequencing used only to triage candidates for individual validation; reported data is a handful of purified variants, not library-wide.</t>
         </is>

</xml_diff>

<commit_message>
Record Vanella 2024 as an open lead
The EP-Seq activity-stability paper behind Vanella 2026. Its DAOx
construct is the one already established for the shipped datasets, so
Phase 3 is settled before it starts, and it is the paper that actually
measured the surface-display expression scores excluded from Vanella
2026 under the wrong authors' name.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FitnessBench_2025_literature_search.xlsx
+++ b/FitnessBench_2025_literature_search.xlsx
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -4935,7 +4935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5106,6 +5106,38 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Vanella 2024 -- the EP-Seq activity-stability paper behind Vanella 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>10.1038/s41467-024-45630-3</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Eighth sweep (2026), found while curating Vanella 2026</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Same DAOx construct as the shipped Vanella 2026 datasets, so Phase 3 is already settled: 365 aa, P80324 1-365, confirmed from the plasmid at Zenodo 10.5281/zenodo.8388902. It is also the paper that actually measured the surface-display expression scores excluded from Vanella 2026, so curating it gives that data a legitimate home under its own authors. Activity-stability tradeoff framing suggests both an activity and a stability readout.</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>Not chased yet. Its supplementary bundle and Zenodo deposit were downloaded during the Vanella 2026 work (record 8388902 includes a 2 GB PacBio FASTQ and a 14 GB Illumina zip -- filter by size). Needs Phase 0-1 from the top.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>